<commit_message>
feat: update FBFS project outputs, restructure embedded files, and enrich knowledge base
- Restructure embedded files: rename CTS/TDR OLE attachments, add SVP plan, product description PPTX, raw extraction dirs
- Update CTS/TDR docx, analysis outputs (README, special characteristics, quality targets, missing items tracker)
- Add new analysis deliverables: exception list, capability declaration template, risk prompt list
- Add 交付物 output directory and 记录 records directory
- Add gen_feasibility_letter.py script for feasibility letter generation
- Enrich knowledge base: fuel-line component knowledge, Stellantis OEM requirements, combo knowledge

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/FBFS/out/分析/客户交付物需求清单.xlsx
+++ b/project/FBFS/out/分析/客户交付物需求清单.xlsx
@@ -29,11 +29,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -45,7 +43,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -55,17 +63,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
+        <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -83,48 +81,37 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -494,16 +481,16 @@
   <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -558,11 +545,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Native Unigraphics and Team Center capability</t>
         </is>
@@ -577,44 +564,40 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>❌ 不可生成</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>需专业工程软件（UG/TcAE）</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Stellantis硬性要求</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 部分生成</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>需要真实UG/TcAE能力信息</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>无（自主生成）</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>待生成</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>AI可生成能力声明框架，需工程师填写实际能力</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Co-design cost breakdown (ED&amp;D)</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Codesign cost breakdown (ED&amp;D)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -627,42 +610,38 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>⚠️ 部分生成</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>核心成本数字需工程师输入</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>需要实际成本数字</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>L2_TDR_ED&amp;D成本模板.xlsx</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>可生成模板框架</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>AI填充框架和项目信息，成本数字需财务填写</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Supplier development team (SDT)</t>
         </is>
@@ -677,44 +656,40 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>⚠️ 部分生成</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>人员名单需工程师填写</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>L2_CTS_SDT团队名册模板.xlsx</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>需要实际人员信息</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>L2_TDR_SDT团队名册模板.xlsx</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>可生成模板框架</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>AI填充模板框架，人员姓名/邮箱需人工填写</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Components add-on (development cost inclusion)</t>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Components add-on (materials for test)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -727,44 +702,40 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>⚠️ 部分生成</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>测试/样件成本需工程师估算</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>L2_CTS_BOM清单模板.xlsx</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>需要实际BOM和成本数据</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>L2_TDR_BOM清单模板.xlsx</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>需列出测试配套件和开发成本</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>AI可列出已知BOM项目，数量/价格需工程师确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Supplier timing related to vehicle planning</t>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Supplier timing (related to vehicle planning)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -777,42 +748,38 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>⚠️ 部分生成</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>SOP/TKO日期未提供</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>无（需自制）</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>待生成</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>⚠️缺口：需向客户索要VP/PS/TKO/SOP日期</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>❌ 不可生成</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>需要工程师评估和客户VP/PS/SOP时间节点</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>强依赖客户提供的车辆开发计划（未提供）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>List of exception</t>
         </is>
@@ -827,42 +794,38 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>✅ 可生成</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>L2_CTS_例外事项清单模板.xlsx</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 部分生成</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>需工程师判断哪些是真实例外</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>L2_TDR_例外事项清单模板.xlsx</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>基于技术评估生成例外清单</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>AI可识别潜在例外项，最终判断由工程师确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>RASI</t>
         </is>
@@ -877,44 +840,40 @@
           <t>SUPPLIER+APPROVAL</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>✅ 可生成</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>L2_CTS_RASI矩阵模板.xlsx</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 部分生成</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>需要确认SI Level和实际职责分工</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>L2_TDR_RASI矩阵模板.xlsx</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>按SI Level填写对应列</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>AI填充Level 2对应列，具体负责人需工程师确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>CAD data for soft tooling prototype</t>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CAD data for soft tooling prototype / CAD at nomination</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -927,44 +886,40 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>❌ 不可生成</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>需3D CAD软件操作</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>需3D CAD软件（UG/NX）</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>概念布局CAD数据</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>属于工程作业，不适合AI生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Complete 2D Drawings (by TKO)</t>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Complete 2D Drawings</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -977,42 +932,38 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>❌ 不可生成</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>需3D CAD软件出2D图纸</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>需CAD工具和工程判断</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>TKO前完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>需TKO前完成，不适合AI生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Best practices sharing</t>
         </is>
@@ -1027,44 +978,40 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>✅ 可生成</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 部分生成</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>需要真实工程经验</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>无（自主生成）</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>基于组织经验库生成</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>AI可基于知识库生成最佳实践框架，需工程师审阅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Product and Process FMEA (by TKO)</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; Process FMEA</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1077,42 +1024,38 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>❌ 不可生成</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>需工程判断</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>需工程判断（失效模式分析）</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>可提供初稿框架参考</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>核心工程文件，AI不做工程判断</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>CAD data at nomination</t>
         </is>
@@ -1127,42 +1070,38 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>❌ 不可生成</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>需3D CAD软件操作</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>需3D CAD软件</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Nomination后完整CAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>与#8同类</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>System performance analysis support</t>
         </is>
@@ -1177,44 +1116,40 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>❌ 不可生成</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>需工程判断+物理测试数据</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>需系统级工程分析</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>配合OEM系统分析</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>需要具体车辆数据和分析工具</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>DV and PV plan (DVP&amp;R)</t>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>DV and PV plan</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1227,42 +1162,34 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>✅ 可生成</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>STLA-DVPR模板.xlsx</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>L2_CTS_SVP验证计划模板.xlsx / STLA-DVPR模板.xlsx</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>待生成</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>基于PF.90197 Annex A生成</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>基于PF.90197 Annex A自动填充</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Support for SOP in assembly plant</t>
         </is>
@@ -1277,34 +1204,30 @@
           <t>SUPPLIER</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>❌ 不可生成</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>需现场物理操作</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>需物理操作和现场支持</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>跳过（不可生成）</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>SOP阶段装配厂现场支持</t>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>跳过</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>现场活动，AI无法生成</t>
         </is>
       </c>
     </row>

</xml_diff>